<commit_message>
up mượn trả sách
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/Import.xlsx
+++ b/src/main/resources/templates/Import.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14904" windowHeight="4392"/>
+    <workbookView windowWidth="13128" windowHeight="4392"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
   <si>
     <t>STT</t>
   </si>
@@ -53,88 +53,70 @@
     <t>Mô tả</t>
   </si>
   <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>Xàm ngôn</t>
-  </si>
-  <si>
-    <t>Ngôn lù</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siêu cấp ngôn lù </t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 2</t>
-  </si>
-  <si>
-    <t>Ngôn lù 2</t>
-  </si>
-  <si>
-    <t>L3</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 3</t>
-  </si>
-  <si>
-    <t>Ngôn lù 3</t>
-  </si>
-  <si>
-    <t>L4</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 4</t>
-  </si>
-  <si>
-    <t>Ngôn lù 4</t>
-  </si>
-  <si>
-    <t>L6</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 6</t>
-  </si>
-  <si>
-    <t>Ngôn lù 6</t>
-  </si>
-  <si>
-    <t>L7</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 7</t>
-  </si>
-  <si>
-    <t>Ngôn lù 7</t>
-  </si>
-  <si>
-    <t>L8</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 8</t>
-  </si>
-  <si>
-    <t>Ngôn lù 8</t>
-  </si>
-  <si>
-    <t>L9</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 9</t>
-  </si>
-  <si>
-    <t>Ngôn lù 9</t>
-  </si>
-  <si>
-    <t>L10</t>
-  </si>
-  <si>
-    <t>Xàm ngôn 10</t>
-  </si>
-  <si>
-    <t>Ngôn lù 10</t>
+    <t>JI1</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 1</t>
+  </si>
+  <si>
+    <t>Phạm Tu</t>
+  </si>
+  <si>
+    <t>quả khế</t>
+  </si>
+  <si>
+    <t>JI2</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 2</t>
+  </si>
+  <si>
+    <t>JI3</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 3</t>
+  </si>
+  <si>
+    <t>JI4</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 4</t>
+  </si>
+  <si>
+    <t>JI5</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 5</t>
+  </si>
+  <si>
+    <t>JI6</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 6</t>
+  </si>
+  <si>
+    <t>JI7</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 7</t>
+  </si>
+  <si>
+    <t>JI8</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 8</t>
+  </si>
+  <si>
+    <t>JI9</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 9</t>
+  </si>
+  <si>
+    <t>JI10</t>
+  </si>
+  <si>
+    <t>Ăn quả nhớ kẻ 10</t>
   </si>
 </sst>
 </file>
@@ -1318,7 +1300,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1330,10 +1312,10 @@
         <v>10</v>
       </c>
       <c r="E2">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -1344,7 +1326,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3">
-        <v>2</v>
+        <v>2001</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
@@ -1353,13 +1335,13 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E3">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>501</v>
+        <v>201</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -1370,22 +1352,22 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4">
-        <v>3</v>
+        <v>2002</v>
       </c>
       <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E4">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="F4">
-        <v>502</v>
+        <v>202</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -1396,22 +1378,22 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5">
-        <v>4</v>
+        <v>2003</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>503</v>
+        <v>-203</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -1422,22 +1404,22 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
-        <v>5</v>
+        <v>2004</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
       </c>
       <c r="E6">
-        <v>-10</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>-10</v>
+        <v>204</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -1448,22 +1430,22 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
-        <v>6</v>
+        <v>2005</v>
       </c>
       <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>505</v>
+        <v>205</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -1474,22 +1456,22 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8">
-        <v>7</v>
+        <v>2006</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E8">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="F8">
-        <v>506</v>
+        <v>206</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -1500,22 +1482,22 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9">
-        <v>8</v>
+        <v>2007</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E9">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="F9">
-        <v>507</v>
+        <v>207</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -1526,22 +1508,22 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10">
-        <v>9</v>
+        <v>2008</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="F10">
-        <v>508</v>
+        <v>208</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -1552,22 +1534,22 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11">
+        <v>2009</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
-        <v>35</v>
-      </c>
       <c r="E11">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="F11">
-        <v>509</v>
+        <v>209</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>

</xml_diff>